<commit_message>
update login form 4.6.2026
</commit_message>
<xml_diff>
--- a/docs/Apptienganh-Tong-Hop.xlsx
+++ b/docs/Apptienganh-Tong-Hop.xlsx
@@ -6,7 +6,10 @@
     <sheet name="Stack" sheetId="1" r:id="rId1"/>
     <sheet name="Trang_APP" sheetId="2" r:id="rId2"/>
     <sheet name="API_Routes" sheetId="3" r:id="rId3"/>
-    <sheet name="Lib_AI_Chinh" sheetId="4" r:id="rId4"/>
+    <sheet name="Components" sheetId="4" r:id="rId4"/>
+    <sheet name="Lib_Chinh" sheetId="5" r:id="rId5"/>
+    <sheet name="Scripts" sheetId="6" r:id="rId6"/>
+    <sheet name="SQL_Schema" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -400,10 +403,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,7 +438,7 @@
         <v>Ngôn ngữ</v>
       </c>
       <c r="B4" t="str">
-        <v>JavaScript (.js/.jsx) + TypeScript (.ts) trong lib/ai</v>
+        <v>JavaScript (.js/.jsx) + TypeScript (.ts/.tsx)</v>
       </c>
     </row>
     <row r="5">
@@ -443,7 +446,7 @@
         <v>API</v>
       </c>
       <c r="B5" t="str">
-        <v>Route Handlers app/api/*/route.js</v>
+        <v>Route Handlers app/api/**/route.{js,ts}</v>
       </c>
     </row>
     <row r="6">
@@ -456,10 +459,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Cache AI</v>
+        <v>Cache</v>
       </c>
       <c r="B7" t="str">
-        <v>Redis (ioredis) + fallback bộ nhớ</v>
+        <v>Redis (ioredis) + bộ nhớ (runtime-settings, AI cache)</v>
       </c>
     </row>
     <row r="8">
@@ -467,7 +470,7 @@
         <v>AI</v>
       </c>
       <c r="B8" t="str">
-        <v>OpenAI Chat Completions + prompt/routing lib/ai</v>
+        <v>OpenAI + prompt/routing lib/ai; fallback dịch MyMemory</v>
       </c>
     </row>
     <row r="9">
@@ -475,39 +478,47 @@
         <v>Speech</v>
       </c>
       <c r="B9" t="str">
-        <v>Azure Speech SDK + Web Speech API (trình duyệt)</v>
+        <v>Azure Speech SDK + Web Speech API</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Email/SMS</v>
+        <v>Thanh toán</v>
       </c>
       <c r="B10" t="str">
-        <v>SendGrid, Nodemailer, Twilio</v>
+        <v>Stripe</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Email/SMS</v>
+      </c>
+      <c r="B11" t="str">
+        <v>SendGrid, Nodemailer, Twilio</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Tên package</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>kids-english-nextjs</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C15"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="41.83203125" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -518,7 +529,7 @@
         <v>File</v>
       </c>
       <c r="C1" t="str">
-        <v>Mô tả gợi ý</v>
+        <v>Mô tả</v>
       </c>
     </row>
     <row r="2">
@@ -534,57 +545,57 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>/vocabulary</v>
+        <v>/auth</v>
       </c>
       <c r="B3" t="str">
-        <v>app/vocabulary/page.js</v>
+        <v>app/auth/page.js</v>
       </c>
       <c r="C3" t="str">
-        <v>Từ vựng + phát âm</v>
+        <v>Đăng nhập / OTP</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>/dictionary</v>
+        <v>/dashboard</v>
       </c>
       <c r="B4" t="str">
-        <v>app/dictionary/page.js</v>
+        <v>app/dashboard/page.js</v>
       </c>
       <c r="C4" t="str">
-        <v>Tra từ điển</v>
+        <v>Tiến độ / dashboard</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>/matching</v>
+        <v>/lessons</v>
       </c>
       <c r="B5" t="str">
-        <v>app/matching/page.js</v>
+        <v>app/lessons/page.js</v>
       </c>
       <c r="C5" t="str">
-        <v>Ghép từ và hình</v>
+        <v>Bài học + chat AI</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>/lessons</v>
+        <v>/quiz</v>
       </c>
       <c r="B6" t="str">
-        <v>app/lessons/page.js</v>
+        <v>app/quiz/page.js (+ quiz.css, error.js)</v>
       </c>
       <c r="C6" t="str">
-        <v>Bài học + chat AI</v>
+        <v>Quiz</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>/quiz</v>
+        <v>/matching</v>
       </c>
       <c r="B7" t="str">
-        <v>app/quiz/page.js</v>
+        <v>app/matching/page.js</v>
       </c>
       <c r="C7" t="str">
-        <v>Quiz</v>
+        <v>Nối từ / ghép hình</v>
       </c>
     </row>
     <row r="8">
@@ -600,55 +611,99 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>/auth</v>
+        <v>/vocabulary</v>
       </c>
       <c r="B9" t="str">
-        <v>app/auth/page.js</v>
+        <v>app/vocabulary/page.js</v>
       </c>
       <c r="C9" t="str">
-        <v>Đăng nhập / OTP</v>
+        <v>Từ vựng</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>/dashboard</v>
+        <v>/dictionary</v>
       </c>
       <c r="B10" t="str">
-        <v>app/dashboard/page.js</v>
+        <v>app/dictionary/page.js (+ layout.js)</v>
       </c>
       <c r="C10" t="str">
-        <v>Dashboard</v>
+        <v>Từ điển</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>/billing/success</v>
+      </c>
+      <c r="B11" t="str">
+        <v>app/billing/success/page.jsx</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Sau thanh toán Stripe</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>/admin</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v>app/admin/page.js</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C12" t="str">
         <v>Quản trị</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>/admin/options</v>
+      </c>
+      <c r="B13" t="str">
+        <v>app/admin/options/page.js</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Cấu hình app</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>/admin/students</v>
+      </c>
+      <c r="B14" t="str">
+        <v>app/admin/students/page.jsx</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Học viên</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>/admin/payments</v>
+      </c>
+      <c r="B15" t="str">
+        <v>app/admin/payments/page.jsx</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Thanh toán (admin)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B42"/>
   <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Endpoint</v>
+        <v>Phương thức / Endpoint</v>
       </c>
       <c r="B1" t="str">
         <v>File</v>
@@ -656,111 +711,111 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>POST /api/auth/login</v>
+        <v>— Auth —</v>
       </c>
       <c r="B2" t="str">
-        <v>app/api/auth/login/route.js</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>POST /api/auth/logout</v>
+        <v>POST</v>
       </c>
       <c r="B3" t="str">
-        <v>app/api/auth/logout/route.js</v>
+        <v>app/api/auth/login/route.js</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>POST /api/auth/register</v>
+        <v>POST</v>
       </c>
       <c r="B4" t="str">
-        <v>app/api/auth/register/route.js</v>
+        <v>app/api/auth/logout/route.js</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>POST /api/auth/request-otp</v>
+        <v>POST</v>
       </c>
       <c r="B5" t="str">
-        <v>app/api/auth/request-otp/route.js</v>
+        <v>app/api/auth/register/route.js</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GET /api/auth/me</v>
+        <v>POST</v>
       </c>
       <c r="B6" t="str">
-        <v>app/api/auth/me/route.js</v>
+        <v>app/api/auth/request-otp/route.js</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GET/POST /api/vocabulary</v>
+        <v>POST</v>
       </c>
       <c r="B7" t="str">
-        <v>app/api/vocabulary/route.js</v>
+        <v>app/api/auth/otp/send/route.ts</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GET /api/vocabulary/topics</v>
+        <v>POST</v>
       </c>
       <c r="B8" t="str">
-        <v>app/api/vocabulary/topics/route.js</v>
+        <v>app/api/auth/otp/verify/route.ts</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GET /api/lessons</v>
+        <v>GET</v>
       </c>
       <c r="B9" t="str">
-        <v>app/api/lessons/route.js</v>
+        <v>app/api/auth/me/route.js</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>POST /api/lessons/chat</v>
+        <v>GET/PATCH</v>
       </c>
       <c r="B10" t="str">
-        <v>app/api/lessons/chat/route.js</v>
+        <v>app/api/auth/profile/route.ts</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>POST /api/translate</v>
+        <v>POST</v>
       </c>
       <c r="B11" t="str">
-        <v>app/api/translate/route.js</v>
+        <v>app/api/auth/profile/avatar/route.ts</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GET /api/dictionary/lookup</v>
+        <v>— Nội dung học —</v>
       </c>
       <c r="B12" t="str">
-        <v>app/api/dictionary/lookup/route.js</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>GET /api/pronunciation/token</v>
+        <v>GET (+POST)</v>
       </c>
       <c r="B13" t="str">
-        <v>app/api/pronunciation/token/route.js</v>
+        <v>app/api/vocabulary/route.js</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>GET /api/matching/round</v>
+        <v>GET</v>
       </c>
       <c r="B14" t="str">
-        <v>app/api/matching/round/route.js</v>
+        <v>app/api/vocabulary/topics/route.js</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>GET /api/quiz/round</v>
+        <v>GET</v>
       </c>
       <c r="B15" t="str">
         <v>app/api/quiz/round/route.js</v>
@@ -768,70 +823,365 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>GET /api/questions</v>
+        <v>GET</v>
       </c>
       <c r="B16" t="str">
-        <v>app/api/questions/route.js</v>
+        <v>app/api/matching/round/route.js</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GET/POST /api/progress</v>
+        <v>GET</v>
       </c>
       <c r="B17" t="str">
-        <v>app/api/progress/route.js</v>
+        <v>app/api/questions/route.js</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GET /api/progress/students</v>
+        <v>GET (+POST)</v>
       </c>
       <c r="B18" t="str">
-        <v>app/api/progress/students/route.js</v>
+        <v>app/api/lessons/route.js</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>GET/POST /api/admin/students</v>
+        <v>POST</v>
       </c>
       <c r="B19" t="str">
-        <v>app/api/admin/students/route.js</v>
+        <v>app/api/lessons/chat/route.js</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>GET /api/admin/students/progress</v>
+        <v>GET</v>
       </c>
       <c r="B20" t="str">
-        <v>app/api/admin/students/progress/route.js</v>
+        <v>app/api/dictionary/lookup/route.js</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>POST /api/admin/import-vocabulary</v>
+        <v>POST</v>
       </c>
       <c r="B21" t="str">
+        <v>app/api/translate/route.js</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>GET</v>
+      </c>
+      <c r="B22" t="str">
+        <v>app/api/pronunciation/token/route.js</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>— Tiến độ —</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>GET/POST</v>
+      </c>
+      <c r="B24" t="str">
+        <v>app/api/progress/route.js</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>GET</v>
+      </c>
+      <c r="B25" t="str">
+        <v>app/api/progress/students/route.js</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>— Admin —</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>GET/POST</v>
+      </c>
+      <c r="B27" t="str">
+        <v>app/api/admin/students/route.js</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>GET</v>
+      </c>
+      <c r="B28" t="str">
+        <v>app/api/admin/students/progress/route.js</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>GET</v>
+      </c>
+      <c r="B29" t="str">
+        <v>app/api/admin/payments/route.ts</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B30" t="str">
+        <v>app/api/admin/payments/confirm/route.ts</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B31" t="str">
         <v>app/api/admin/import-vocabulary/route.js</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>GET/PATCH</v>
+      </c>
+      <c r="B32" t="str">
+        <v>app/api/admin/app-settings/route.ts</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>— Thanh toán —</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B34" t="str">
+        <v>app/api/payments/create/route.ts</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B35" t="str">
+        <v>app/api/payments/confirm/route.ts</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B36" t="str">
+        <v>app/api/billing/checkout/route.ts</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B37" t="str">
+        <v>app/api/billing/webhook/route.ts</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B38" t="str">
+        <v>app/api/billing/verify-session/route.ts</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>POST</v>
+      </c>
+      <c r="B39" t="str">
+        <v>app/api/billing/track/route.ts</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>— Hệ thống —</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>GET</v>
+      </c>
+      <c r="B41" t="str">
+        <v>app/api/health/route.ts</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>GET</v>
+      </c>
+      <c r="B42" t="str">
+        <v>app/api/health/db/route.ts</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B42"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <cols>
-    <col min="1" max="1" width="41.83203125" customWidth="1"/>
-    <col min="2" max="2" width="54.83203125" customWidth="1"/>
+    <col min="1" max="1" width="45.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Đường dẫn</v>
+        <v>File</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Ghi chú</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>components/KidMainNav.jsx</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Menu chính</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>components/DictionarySearchBar.jsx</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Ô tra từ trên header</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>components/AppProviders.jsx</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Providers app</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>components/GuestGateProvider.jsx</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Gate khách</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>components/HeaderProfile.jsx</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Avatar / menu tài khoản</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>components/TrialCountdown.jsx</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Đếm trial</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>components/account/AccountModal.jsx</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Modal tài khoản</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>components/account/BottomAccountDock.jsx</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Dock đăng nhập</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>components/billing/UpgradeMenu.jsx</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Nâng cấp</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>components/billing/PaywallProvider.jsx</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Paywall context</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>components/billing/PaywallModal.jsx</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Modal paywall</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>components/billing/ServicePackagesModal.jsx</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Gói dịch vụ</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>components/billing/BankTransferModal.jsx</v>
+      </c>
+      <c r="B14" t="str">
+        <v>CK ngân hàng</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B13"/>
+  <cols>
+    <col min="1" max="1" width="33.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>File / thư mục</v>
       </c>
       <c r="B1" t="str">
         <v>Vai trò</v>
@@ -839,82 +1189,280 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>lib/ai/client.ts</v>
+        <v>lib/db.js</v>
       </c>
       <c r="B2" t="str">
-        <v>completeAi, cache, gọi OpenAI</v>
+        <v>MySQL pool</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>lib/ai/router.ts</v>
+        <v>lib/auth.js</v>
       </c>
       <c r="B3" t="str">
-        <v>Chọn model / maxTokens / temperature theo route type</v>
+        <v>Session / cookie</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>lib/ai/prompts/</v>
+        <v>lib/auth/create-session.ts</v>
       </c>
       <c r="B4" t="str">
-        <v>chat, translate, grammar, speaking (TS)</v>
+        <v>Tạo session</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>lib/ai/experiments/chat-prompt-ab.ts</v>
+        <v>middleware.ts</v>
       </c>
       <c r="B5" t="str">
-        <v>A/B test prompt chat + metrics MySQL</v>
+        <v>Bảo vệ route + API</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>lib/ai/cache/response-cache.ts</v>
+        <v>lib/http/api-guards.js</v>
       </c>
       <c r="B6" t="str">
-        <v>Redis + memory fallback</v>
+        <v>Guard API</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>lib/ai/services/lessons-chat.service.js</v>
+        <v>lib/http/ai-entitlement.ts</v>
       </c>
       <c r="B7" t="str">
-        <v>Chat bài học (JSON tutor)</v>
+        <v>Hạn mức AI / gói</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>lib/ai/services/translate.service.js</v>
+        <v>lib/subscriptions/</v>
       </c>
       <c r="B8" t="str">
-        <v>Dịch EN→VI</v>
+        <v>Subscription service</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>lib/db.js</v>
+        <v>lib/billing/</v>
       </c>
       <c r="B9" t="str">
-        <v>Kết nối MySQL pool</v>
+        <v>Stripe, checkout, webhook xử lý</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>lib/auth.js</v>
+        <v>lib/otp/</v>
       </c>
       <c r="B10" t="str">
-        <v>Xác thực session / OTP</v>
+        <v>OTP service + bảng</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>components/DictionarySearchBar.jsx</v>
+        <v>lib/runtime-settings/</v>
       </c>
       <c r="B11" t="str">
-        <v>Ô tìm từ trên menu</v>
+        <v>Cấu hình Redis/cache</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>lib/vocabulary/ensure-schema.js</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Schema từ vựng</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>lib/ai/</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Router, prompts, services, cache</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="57.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Script</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Mục đích gợi ý</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>scripts/test-db-connection.mjs</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Kiểm tra DB</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>scripts/check-vocab-count.mjs</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Đếm từ vựng</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>scripts/health-check.mjs</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Health</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>scripts/dev-watchdog.mjs</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Watchdog dev</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>scripts/seed-1000-vocabulary.mjs</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Seed từ vựng</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>scripts/export-project-excel.mjs</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Xuất Excel này</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>… (còn ~28 script)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>normalize/backfill/import vocabulary, IPA, câu ví dụ VI</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B11"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>File</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Vị trí</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>database.sql</v>
+      </c>
+      <c r="B2" t="str">
+        <v>gốc dự án</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>database.nextjs.sql</v>
+      </c>
+      <c r="B3" t="str">
+        <v>gốc dự án</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>database.vocabulary.sql</v>
+      </c>
+      <c r="B4" t="str">
+        <v>gốc dự án</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>database.auth.sql</v>
+      </c>
+      <c r="B5" t="str">
+        <v>gốc dự án</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>lib/data/subscriptions.sql</v>
+      </c>
+      <c r="B6" t="str">
+        <v>lib/data</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>lib/data/otp_codes.sql</v>
+      </c>
+      <c r="B7" t="str">
+        <v>lib/data</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>lib/data/payments.sql</v>
+      </c>
+      <c r="B8" t="str">
+        <v>lib/data</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>lib/data/billing_conversion.sql</v>
+      </c>
+      <c r="B9" t="str">
+        <v>lib/data</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>lib/data/chat_prompt_variant_usage.sql</v>
+      </c>
+      <c r="B10" t="str">
+        <v>lib/data</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>lib/data/chat_prompt_ab.sql</v>
+      </c>
+      <c r="B11" t="str">
+        <v>lib/data</v>
       </c>
     </row>
   </sheetData>

</xml_diff>